<commit_message>
refactor(demo): align Card pipeline with new sp.regtable full-coef default
Drop 8 misaligned `keep=["educ"]` filters from the Card (1995) pipeline
so Tables 2/2c/2d/3/A1 (and the corresponding sp.collect bundle entries)
show every estimated parameter — controls AND intercept — per the new
StatsPAI skill convention. The 3 legitimate focal-only uses (IV
first-stage triplet × 2 + interaction-form heterogeneity × 1) are
preserved. Headline numbers unchanged: OLS β=0.075, 2SLS β=0.132,
first-stage F=14.14, Oster δ*=16.4.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-StatsPAI-skill/replication/paper.xlsx
+++ b/demo-StatsPAI-skill/replication/paper.xlsx
@@ -919,7 +919,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>1.3398450009593703e-14</t>
+          <t>1.3398450009593587e-14</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>0.0009115426060092432</t>
+          <t>0.000911542606009244</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>6.981252999887786e-05</t>
+          <t>6.981252999887759e-05</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>3.6730337292298855e-33</t>
+          <t>3.6730337292298636e-33</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>2.6732899123799257e-71</t>
+          <t>2.6732899123800616e-71</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>1.7379969925770925e-131</t>
+          <t>1.7379969925768423e-131</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>3.4012060836764276e-11</t>
+          <t>3.4012060836764296e-11</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
@@ -1213,7 +1213,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>1.3318858250924414e-05</t>
+          <t>1.331885825092444e-05</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
@@ -1261,14 +1261,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1312,27 +1312,27 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>educ</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0.052***</t>
+          <t>5.571***</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0.093***</t>
+          <t>4.469***</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>0.074***</t>
+          <t>4.734***</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>0.075***</t>
+          <t>4.621***</t>
         </is>
       </c>
     </row>
@@ -1340,90 +1340,560 @@
       <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>(0.003)</t>
+          <t>(0.039)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.070)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.070)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.074)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
+          <t>educ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>0.052***</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0.093***</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>0.074***</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>0.075***</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>(0.003)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>exper</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr"/>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0.090***</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>0.084***</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>0.085***</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>(0.007)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>(0.007)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>(0.007)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>expersq</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr"/>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr"/>
+      <c r="C13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>-0.190***</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-0.199***</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr"/>
+      <c r="C14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr"/>
+      <c r="C15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>-0.125***</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-0.148***</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>(0.015)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>(0.028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>smsa</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>0.161***</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>0.136***</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr"/>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>(0.015)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>smsa66</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr"/>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="5" t="inlineStr"/>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>0.026</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr"/>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="5" t="inlineStr"/>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>reg662</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="5" t="inlineStr"/>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>0.096***</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr"/>
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="5" t="inlineStr"/>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>(0.035)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>reg663</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>0.145***</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>reg664</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0.055</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>reg665</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr"/>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="5" t="inlineStr"/>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>0.128***</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr"/>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="5" t="inlineStr"/>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>(0.043)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>reg666</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr"/>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="5" t="inlineStr"/>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0.141***</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr"/>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="5" t="inlineStr"/>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>(0.045)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>reg667</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr"/>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr"/>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>0.118***</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr"/>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>(0.046)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>reg668</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>-0.056</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>(0.051)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>reg669</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>0.119***</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>(0.039)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>3,010</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>3,010</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>3,010</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>3,010</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>R²</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>0.099</t>
         </is>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C38" s="7" t="inlineStr">
         <is>
           <t>0.196</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>0.291</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E38" s="7" t="inlineStr">
         <is>
           <t>0.300</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Standard errors in parentheses</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>* p&lt;0.10, ** p&lt;0.05, *** p&lt;0.01</t>
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>*** p&lt;0.01, ** p&lt;0.05, * p&lt;0.10</t>
         </is>
       </c>
     </row>
@@ -1639,7 +2109,7 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>* p&lt;0.10, ** p&lt;0.05, *** p&lt;0.01</t>
+          <t>*** p&lt;0.01, ** p&lt;0.05, * p&lt;0.10</t>
         </is>
       </c>
     </row>
@@ -1654,16 +2124,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1726,42 +2196,42 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>educ</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0.074***</t>
+          <t>4.734***</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0.071***</t>
+          <t>2.476***</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>0.074***</t>
+          <t>4.686***</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>0.259</t>
+          <t>231844238082004.656</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>0.070***</t>
+          <t>4.762***</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>0.075***</t>
+          <t>2.425***</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>0.070***</t>
+          <t>4.867***</t>
         </is>
       </c>
     </row>
@@ -1769,219 +2239,699 @@
       <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.070)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>(0.008)</t>
+          <t>(0.075)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.079)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>()</t>
+          <t>(4141688650879277203456.000)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>(0.005)</t>
+          <t>(0.089)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.043)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>(0.007)</t>
+          <t>(0.126)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>educ</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>3,010</t>
+          <t>0.074***</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>0.071***</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>2,307</t>
+          <t>0.074***</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>1,215</t>
+          <t>0.259</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>1,795</t>
+          <t>0.070***</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>2,146</t>
+          <t>0.075***</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>864</t>
+          <t>0.070***</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>R²</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="inlineStr"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>0.291</t>
+          <t>(0.004)</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>0.266</t>
+          <t>(0.008)</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>0.216</t>
+          <t>(0.004)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>-0.609</t>
+          <t>()</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>0.187</t>
+          <t>(0.005)</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>0.233</t>
+          <t>(0.004)</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>0.294</t>
+          <t>(0.007)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
+          <t>exper</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>0.084***</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>0.034**</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>0.090***</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>0.327</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>0.087***</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>0.089***</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>0.068***</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>(0.007)</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>(0.014)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>(0.008)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>(137363.606)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>(0.009)</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>(0.009)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>(0.010)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>expersq</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-0.001</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>-0.009</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>(0.001)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>(8955.173)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>-0.190***</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2.476***</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-0.049</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>-0.123***</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>-0.175***</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>-0.231***</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>(0.075)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>()</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>()</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>(0.029)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>(0.021)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>-0.125***</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>-0.214***</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>-0.100***</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-231844238082004.094</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>-0.125***</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>-0.114***</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>(0.015)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>(6047170633136027467776.000)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>(0.029)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>smsa</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>0.161***</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0.143***</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>0.155***</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>0.184***</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>0.153***</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>2.425***</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>(0.015)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>(0.033)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>(0.032)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>(0.021)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>(0.043)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>3,010</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>2,307</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>1,215</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>1,795</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>2,146</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>864</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>R²</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>0.291</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>0.266</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>0.216</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>-0.607</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>0.187</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>0.233</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>0.294</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Adj. R²</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B21" s="5" t="inlineStr">
         <is>
           <t>0.289</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>0.260</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>0.214</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>-0.617</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>-0.615</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
         <is>
           <t>0.185</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>0.231</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H21" s="5" t="inlineStr">
         <is>
           <t>0.289</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>204.932</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>42.099</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>105.401</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
-        <is>
-          <t>-76.191</t>
-        </is>
-      </c>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>-76.060</t>
+        </is>
+      </c>
+      <c r="F22" s="7" t="inlineStr">
         <is>
           <t>68.674</t>
         </is>
       </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="G22" s="7" t="inlineStr">
         <is>
           <t>108.488</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H22" s="7" t="inlineStr">
         <is>
           <t>59.603</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Standard errors in parentheses</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t>* p&lt;0.10, ** p&lt;0.05, *** p&lt;0.01</t>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>*** p&lt;0.01, ** p&lt;0.05, * p&lt;0.10</t>
         </is>
       </c>
     </row>
@@ -1996,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:K52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2089,52 +3039,52 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>educ</t>
+          <t>Intercept</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0.075***</t>
+          <t>4.621***</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>0.074***</t>
+          <t>4.524***</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>0.069***</t>
+          <t>4.741***</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>0.072***</t>
+          <t>4.695***</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>0.071***</t>
+          <t>2.476***</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>0.074***</t>
+          <t>4.686***</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>0.070***</t>
+          <t>4.379***</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>0.132**</t>
+          <t>3.666***</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>0.157***</t>
+          <t>3.237***</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr"/>
@@ -2143,47 +3093,47 @@
       <c r="A6" s="4" t="inlineStr"/>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.074)</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>(0.005)</t>
+          <t>(0.088)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.072)</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.072)</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>(0.008)</t>
+          <t>(0.075)</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>(0.004)</t>
+          <t>(0.079)</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>(0.005)</t>
+          <t>(0.112)</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>(0.054)</t>
+          <t>(0.911)</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
-          <t>(0.053)</t>
+          <t>(0.884)</t>
         </is>
       </c>
       <c r="K6" s="5" t="inlineStr"/>
@@ -2191,45 +3141,101 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>First-stage F</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr"/>
-      <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
-      <c r="G7" s="5" t="inlineStr"/>
-      <c r="H7" s="5" t="inlineStr"/>
+          <t>educ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>0.075***</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>0.074***</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>0.069***</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>0.072***</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>0.071***</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>0.074***</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>0.070***</t>
+        </is>
+      </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>13.26</t>
+          <t>0.132**</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>7.89</t>
+          <t>0.157***</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Hansen J p-value</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr"/>
-      <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5" t="inlineStr"/>
-      <c r="F8" s="5" t="inlineStr"/>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>(0.005)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>(0.008)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>(0.005)</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>(0.054)</t>
+        </is>
+      </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>0.264</t>
+          <t>(0.053)</t>
         </is>
       </c>
       <c r="K8" s="5" t="inlineStr"/>
@@ -2237,109 +3243,101 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>exper</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>3,010</t>
+          <t>0.085***</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>2,220</t>
+          <t>0.090***</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>2,977</t>
+          <t>0.079***</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>2,977</t>
+          <t>0.081***</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>703</t>
+          <t>0.034**</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>2,307</t>
+          <t>0.090***</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>2,061</t>
+          <t>0.095***</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>3,010</t>
+          <t>0.108***</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>3,010</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>3,010</t>
-        </is>
-      </c>
+          <t>0.119***</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>R²</t>
-        </is>
-      </c>
+      <c r="A10" s="4" t="inlineStr"/>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>0.300</t>
+          <t>(0.007)</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>0.274</t>
+          <t>(0.008)</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>0.285</t>
+          <t>(0.007)</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>0.296</t>
+          <t>(0.006)</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>0.266</t>
+          <t>(0.014)</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>0.216</t>
+          <t>(0.008)</t>
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>0.237</t>
+          <t>(0.009)</t>
         </is>
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>0.238</t>
+          <t>(0.023)</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>0.170</t>
+          <t>(0.023)</t>
         </is>
       </c>
       <c r="K10" s="5" t="inlineStr"/>
@@ -2347,104 +3345,1594 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>expersq</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>-0.001</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>-0.003***</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>-0.002***</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>(0.001)</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>(0.000)</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>black</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>-0.199***</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>-0.165***</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>-0.193***</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>-0.189***</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>2.476***</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>-0.148***</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>-0.147***</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>-0.123**</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>(0.025)</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>(0.075)</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>()</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>(0.028)</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>(0.053)</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>(0.052)</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>south</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>-0.148***</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>-0.124***</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>-0.151***</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>-0.143***</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>-0.214***</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>-0.100***</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>-0.100***</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>-0.145***</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>-0.143***</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>(0.028)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>(0.027)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>(0.026)</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>(0.035)</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>(0.029)</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>(0.030)</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>smsa</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>0.136***</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>0.138***</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>0.131***</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>0.130***</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>0.143***</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>0.155***</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>0.123***</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>0.112***</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>0.101***</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>(0.022)</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>(0.033)</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>(0.017)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>(0.023)</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>(0.031)</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="inlineStr">
+        <is>
+          <t>(0.031)</t>
+        </is>
+      </c>
+      <c r="K18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>smsa66</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>0.026</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>0.024</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>0.023</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>0.022</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr"/>
+      <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>0.036</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>0.019</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>0.015</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>(0.019)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>(0.022)</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>(0.018)</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr"/>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>(0.022)</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>(0.021)</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>(0.021)</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>reg662</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>0.096***</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>0.089**</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>0.083**</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>0.095***</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr"/>
+      <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>0.103**</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>0.101***</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>0.103***</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr"/>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>(0.035)</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>(0.042)</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>(0.035)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr"/>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>(0.037)</t>
+        </is>
+      </c>
+      <c r="J22" s="5" t="inlineStr">
+        <is>
+          <t>(0.038)</t>
+        </is>
+      </c>
+      <c r="K22" s="5" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>reg663</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>0.145***</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>0.121***</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>0.139***</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>0.139***</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr"/>
+      <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>0.126***</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>0.148***</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>0.150***</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr"/>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>(0.034)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>(0.033)</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>(0.040)</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>(0.036)</t>
+        </is>
+      </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>(0.037)</t>
+        </is>
+      </c>
+      <c r="K24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>reg664</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>0.055</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>0.039</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>0.053</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>0.049</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr"/>
+      <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>0.049</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>0.050</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>0.048</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr"/>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>(0.048)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>(0.040)</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>(0.047)</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>(0.044)</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>(0.046)</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>reg665</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>0.128***</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>0.095*</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>0.118***</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>0.119***</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr"/>
+      <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>0.124**</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>0.146***</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>0.154***</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr"/>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>(0.043)</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>(0.052)</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>(0.042)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="5" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>(0.053)</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>(0.049)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>(0.051)</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>reg666</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>0.141***</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>0.108*</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>0.136***</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>0.137***</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr"/>
+      <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>0.159***</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>0.163***</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>0.173***</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr"/>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>(0.045)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>(0.056)</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>(0.045)</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>(0.043)</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr"/>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>(0.058)</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>(0.052)</t>
+        </is>
+      </c>
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>(0.054)</t>
+        </is>
+      </c>
+      <c r="K30" s="5" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>reg667</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>0.118***</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>0.101*</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>0.111**</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>0.121***</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr"/>
+      <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>0.091</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>0.135***</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>0.142***</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr"/>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>(0.046)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>(0.054)</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>(0.045)</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>(0.044)</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr"/>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>(0.057)</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>(0.051)</t>
+        </is>
+      </c>
+      <c r="J32" s="5" t="inlineStr">
+        <is>
+          <t>(0.052)</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>reg668</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>-0.056</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>-0.068</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>-0.050</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>-0.051</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>-0.048</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>-0.083</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>-0.095</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr"/>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>(0.051)</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>(0.060)</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>(0.051)</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>(0.048)</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>(0.059)</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>(0.057)</t>
+        </is>
+      </c>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>(0.059)</t>
+        </is>
+      </c>
+      <c r="K34" s="5" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>reg669</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>0.119***</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>0.092**</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>0.101***</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>0.119***</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>0.122***</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>0.108***</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>0.103**</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr"/>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>(0.039)</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>(0.045)</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>(0.038)</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>(0.038)</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>(0.046)</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>(0.041)</t>
+        </is>
+      </c>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>(0.043)</t>
+        </is>
+      </c>
+      <c r="K36" s="5" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>fatheduc</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>-0.001</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="5" t="inlineStr"/>
+      <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr"/>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>(0.003)</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr"/>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>motheduc</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>0.008**</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr"/>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr"/>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr"/>
+      <c r="H40" s="5" t="inlineStr"/>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>IQ</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>0.002***</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr"/>
+      <c r="B42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>(0.001)</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>ATE</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr">
+        <is>
+          <t>0.074***</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr"/>
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="inlineStr">
+        <is>
+          <t>(0.004)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>First-stage F</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr">
+        <is>
+          <t>13.26</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr">
+        <is>
+          <t>7.89</t>
+        </is>
+      </c>
+      <c r="K45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Hansen J p-value</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr">
+        <is>
+          <t>0.264</t>
+        </is>
+      </c>
+      <c r="K46" s="5" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>3,010</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>2,220</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>2,977</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>2,977</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>703</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>2,307</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>2,061</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr">
+        <is>
+          <t>3,010</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr">
+        <is>
+          <t>3,010</t>
+        </is>
+      </c>
+      <c r="K47" s="5" t="inlineStr">
+        <is>
+          <t>3,010</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>R²</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>0.300</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>0.274</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>0.285</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>0.296</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>0.266</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>0.216</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>0.237</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>0.238</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr">
+        <is>
+          <t>0.170</t>
+        </is>
+      </c>
+      <c r="K48" s="5" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
           <t>Adj. R²</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>0.296</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>0.269</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>0.281</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>0.292</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F49" s="5" t="inlineStr">
         <is>
           <t>0.260</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G49" s="5" t="inlineStr">
         <is>
           <t>0.214</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H49" s="5" t="inlineStr">
         <is>
           <t>0.231</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr"/>
-      <c r="K11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B50" s="7" t="inlineStr">
         <is>
           <t>85.476</t>
         </is>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C50" s="7" t="inlineStr">
         <is>
           <t>48.967</t>
         </is>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>78.534</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E50" s="7" t="inlineStr">
         <is>
           <t>83.021</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="F50" s="7" t="inlineStr">
         <is>
           <t>42.099</t>
         </is>
       </c>
-      <c r="G12" s="7" t="inlineStr">
+      <c r="G50" s="7" t="inlineStr">
         <is>
           <t>105.401</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="H50" s="7" t="inlineStr">
         <is>
           <t>39.663</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr"/>
-      <c r="J12" s="7" t="inlineStr"/>
-      <c r="K12" s="7" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="I50" s="7" t="inlineStr"/>
+      <c r="J50" s="7" t="inlineStr"/>
+      <c r="K50" s="7" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
         <is>
           <t>Standard errors in parentheses</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>* p&lt;0.10, ** p&lt;0.05, *** p&lt;0.01</t>
+    <row r="52">
+      <c r="A52" s="8" t="inlineStr">
+        <is>
+          <t>*** p&lt;0.01, ** p&lt;0.05, * p&lt;0.10</t>
         </is>
       </c>
     </row>

</xml_diff>